<commit_message>
doc: add notes and files for daily lecture
- add hmi screens and ladder logic
- add notes + cleaned-notes
- update plc io map csv
</commit_message>
<xml_diff>
--- a/plc/plc-io-map.xlsx
+++ b/plc/plc-io-map.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_최예현\intel26\plc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_se4n\intel26\plc\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -154,15 +154,6 @@
     <t>SOL2</t>
   </si>
   <si>
-    <t>SOL3</t>
-  </si>
-  <si>
-    <t>SOL4</t>
-  </si>
-  <si>
-    <t>SOL5</t>
-  </si>
-  <si>
     <t>SOL6</t>
   </si>
   <si>
@@ -424,6 +415,18 @@
   </si>
   <si>
     <t>가공</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SOL5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SOL3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SOL4</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -431,7 +434,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -795,6 +798,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -815,9 +821,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1100,7 +1103,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="E2:K23"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="5" max="5" width="12.125" customWidth="1"/>
     <col min="6" max="6" width="15.125" customWidth="1"/>
@@ -1110,20 +1113,20 @@
     <col min="11" max="11" width="14.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E2" s="33" t="s">
+    <row r="2" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
+      <c r="E2" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="36" t="s">
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="J2" s="37"/>
-      <c r="K2" s="37"/>
-    </row>
-    <row r="3" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J2" s="38"/>
+      <c r="K2" s="38"/>
+    </row>
+    <row r="3" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1139,23 +1142,23 @@
       <c r="I3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="38" t="s">
+      <c r="J3" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="K3" s="39"/>
-    </row>
-    <row r="4" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K3" s="40"/>
+    </row>
+    <row r="4" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>15</v>
@@ -1164,21 +1167,21 @@
         <v>28</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E5" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>16</v>
@@ -1190,18 +1193,18 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E6" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>17</v>
@@ -1210,18 +1213,18 @@
         <v>33</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E7" s="1" t="s">
         <v>3</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="1" t="s">
@@ -1231,18 +1234,18 @@
         <v>30</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E8" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="1" t="s">
@@ -1252,18 +1255,18 @@
         <v>29</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E9" s="1" t="s">
         <v>5</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="1" t="s">
@@ -1273,18 +1276,18 @@
         <v>32</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H10" s="5"/>
       <c r="I10" s="1" t="s">
@@ -1294,55 +1297,55 @@
         <v>31</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E11" s="1" t="s">
         <v>7</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="1" t="s">
         <v>22</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="K11" s="5"/>
     </row>
-    <row r="12" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E12" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>23</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="K12" s="5"/>
     </row>
-    <row r="13" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="5:11" s="4" customFormat="1" ht="21" customHeight="1">
       <c r="E13" s="1" t="s">
         <v>9</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="5"/>
@@ -1350,41 +1353,41 @@
         <v>24</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="5:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="5:11" ht="18.75" customHeight="1">
       <c r="E14" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G14" s="5"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="5:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="5:11" ht="18.75" customHeight="1">
       <c r="E15" s="1"/>
       <c r="F15" s="5"/>
       <c r="G15" s="5"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="5:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="5:11" ht="18.75" customHeight="1">
       <c r="E16" s="1"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
@@ -1393,24 +1396,24 @@
       <c r="J16" s="5"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="5:11" ht="33" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:11" ht="33">
       <c r="E17" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="F17" s="32" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G17" s="5"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="J17" s="32" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="5:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:11">
       <c r="E18" s="1"/>
       <c r="F18" s="32"/>
       <c r="G18" s="5"/>
@@ -1419,7 +1422,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="5:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:11">
       <c r="E19" s="1"/>
       <c r="F19" s="32"/>
       <c r="G19" s="5"/>
@@ -1428,7 +1431,7 @@
       <c r="J19" s="5"/>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="5:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:11">
       <c r="E20" s="1"/>
       <c r="F20" s="32"/>
       <c r="G20" s="5"/>
@@ -1437,7 +1440,7 @@
       <c r="J20" s="5"/>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="5:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:11">
       <c r="E21" s="1"/>
       <c r="F21" s="32"/>
       <c r="G21" s="5"/>
@@ -1446,7 +1449,7 @@
       <c r="J21" s="5"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="5:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="5:11">
       <c r="E22" s="1"/>
       <c r="F22" s="32"/>
       <c r="G22" s="5"/>
@@ -1455,7 +1458,7 @@
       <c r="J22" s="5"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="5:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="5:11">
       <c r="E23" s="1"/>
       <c r="F23" s="32"/>
       <c r="G23" s="5"/>
@@ -1479,28 +1482,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:Z20"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
   <sheetData>
-    <row r="1" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:26">
       <c r="M1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="2" spans="2:26" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="2:26">
       <c r="C2" s="31" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="M2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="2:26">
+      <c r="C3" s="31" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="C3" s="31" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="2:26" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:26" ht="17.25" thickBot="1"/>
+    <row r="5" spans="2:26">
       <c r="E5" s="9">
         <v>8</v>
       </c>
@@ -1541,24 +1544,24 @@
         <v>1</v>
       </c>
       <c r="X5" s="30" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6" spans="2:26" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="2:26">
       <c r="E6" s="27" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F6" s="28" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G6" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="I6" s="27" t="s">
         <v>49</v>
-      </c>
-      <c r="H6" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="I6" s="27" t="s">
-        <v>52</v>
       </c>
       <c r="J6" s="28" t="s">
         <v>31</v>
@@ -1573,7 +1576,7 @@
         <v>30</v>
       </c>
       <c r="N6" s="28" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="O6" s="28" t="s">
         <v>27</v>
@@ -1585,15 +1588,15 @@
         <v>2</v>
       </c>
       <c r="X6" s="30" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="2:26" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="2:26">
       <c r="E7" s="27" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G7" s="28" t="s">
         <v>24</v>
@@ -1620,7 +1623,7 @@
         <v>17</v>
       </c>
       <c r="O7" s="28" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="P7" s="29" t="s">
         <v>15</v>
@@ -1629,15 +1632,15 @@
         <v>3</v>
       </c>
       <c r="X7" s="30" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8" spans="2:26" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="2:26">
       <c r="B8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
@@ -1695,15 +1698,15 @@
         <v>4</v>
       </c>
       <c r="X8" s="30" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="2:26" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="2:26" ht="17.25" thickBot="1">
       <c r="B9" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E9" s="15">
         <v>0</v>
@@ -1761,41 +1764,41 @@
         <v>5</v>
       </c>
       <c r="X9" s="30" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="2:26" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="2:26">
       <c r="W10" s="7">
         <v>6</v>
       </c>
       <c r="X10" s="30" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="11" spans="2:26" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="2:26">
       <c r="W11" s="7">
         <v>7</v>
       </c>
       <c r="X11" s="30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="2:26">
+      <c r="D12" s="33" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="12" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="D12" s="40" t="s">
-        <v>85</v>
-      </c>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="40"/>
-      <c r="J12" s="40"/>
-      <c r="K12" s="40"/>
-      <c r="L12" s="40"/>
-      <c r="M12" s="40"/>
-      <c r="N12" s="40"/>
-      <c r="O12" s="40"/>
-      <c r="P12" s="40">
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
+      <c r="J12" s="33"/>
+      <c r="K12" s="33"/>
+      <c r="L12" s="33"/>
+      <c r="M12" s="33"/>
+      <c r="N12" s="33"/>
+      <c r="O12" s="33"/>
+      <c r="P12" s="33">
         <v>1</v>
       </c>
       <c r="R12" s="26" t="str">
@@ -1818,16 +1821,16 @@
         <v>8</v>
       </c>
       <c r="X12" s="30" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="Z12" t="str">
         <f>CONCATENATE("MOV H",U12," K3Y20")</f>
         <v>MOV H001 K3Y20</v>
       </c>
     </row>
-    <row r="13" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:26">
       <c r="D13" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="M13">
         <v>1</v>
@@ -1855,33 +1858,33 @@
         <v>9</v>
       </c>
       <c r="X13" s="30" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="Z13" t="str">
         <f t="shared" ref="Z13:Z20" si="4">CONCATENATE("MOV H",U13," K3Y20")</f>
         <v>MOV H008 K3Y20</v>
       </c>
     </row>
-    <row r="14" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="D14" s="40" t="s">
-        <v>87</v>
-      </c>
-      <c r="E14" s="40"/>
-      <c r="F14" s="40">
-        <v>1</v>
-      </c>
-      <c r="G14" s="40"/>
-      <c r="H14" s="40"/>
-      <c r="I14" s="40"/>
-      <c r="J14" s="40"/>
-      <c r="K14" s="40"/>
-      <c r="L14" s="40"/>
-      <c r="M14" s="40"/>
-      <c r="N14" s="40">
-        <v>1</v>
-      </c>
-      <c r="O14" s="40"/>
-      <c r="P14" s="40">
+    <row r="14" spans="2:26">
+      <c r="D14" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33">
+        <v>1</v>
+      </c>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="33"/>
+      <c r="J14" s="33"/>
+      <c r="K14" s="33"/>
+      <c r="L14" s="33"/>
+      <c r="M14" s="33"/>
+      <c r="N14" s="33">
+        <v>1</v>
+      </c>
+      <c r="O14" s="33"/>
+      <c r="P14" s="33">
         <v>0</v>
       </c>
       <c r="R14" s="26" t="str">
@@ -1904,16 +1907,16 @@
         <v>10</v>
       </c>
       <c r="X14" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="Z14" t="str">
         <f t="shared" si="4"/>
         <v>MOV H404 K3Y20</v>
       </c>
     </row>
-    <row r="15" spans="2:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:26">
       <c r="D15" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1944,33 +1947,33 @@
         <v>11</v>
       </c>
       <c r="X15" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="Z15" t="str">
         <f t="shared" si="4"/>
         <v>MOV H402 K3Y20</v>
       </c>
     </row>
-    <row r="16" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="D16" s="40" t="s">
-        <v>89</v>
-      </c>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40">
-        <v>0</v>
-      </c>
-      <c r="G16" s="40"/>
-      <c r="H16" s="40"/>
-      <c r="I16" s="40"/>
-      <c r="J16" s="40"/>
-      <c r="K16" s="40">
-        <v>1</v>
-      </c>
-      <c r="L16" s="40"/>
-      <c r="M16" s="40"/>
-      <c r="N16" s="40"/>
-      <c r="O16" s="40"/>
-      <c r="P16" s="40"/>
+    <row r="16" spans="2:26">
+      <c r="D16" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33">
+        <v>0</v>
+      </c>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="33">
+        <v>1</v>
+      </c>
+      <c r="L16" s="33"/>
+      <c r="M16" s="33"/>
+      <c r="N16" s="33"/>
+      <c r="O16" s="33"/>
+      <c r="P16" s="33"/>
       <c r="R16" s="26" t="str">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1991,16 +1994,16 @@
         <v>12</v>
       </c>
       <c r="X16" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="Z16" t="str">
         <f t="shared" si="4"/>
         <v>MOV H020 K3Y20</v>
       </c>
     </row>
-    <row r="17" spans="4:26" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:26">
       <c r="D17" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2025,33 +2028,33 @@
         <v>13</v>
       </c>
       <c r="X17" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="Z17" t="str">
         <f t="shared" si="4"/>
         <v>MOV H800 K3Y20</v>
       </c>
     </row>
-    <row r="18" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D18" s="40" t="s">
-        <v>91</v>
-      </c>
-      <c r="E18" s="40">
-        <v>0</v>
-      </c>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="40"/>
-      <c r="J18" s="40">
-        <v>1</v>
-      </c>
-      <c r="K18" s="40"/>
-      <c r="L18" s="40"/>
-      <c r="M18" s="40"/>
-      <c r="N18" s="40"/>
-      <c r="O18" s="40"/>
-      <c r="P18" s="40"/>
+    <row r="18" spans="4:26">
+      <c r="D18" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="E18" s="33">
+        <v>0</v>
+      </c>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+      <c r="J18" s="33">
+        <v>1</v>
+      </c>
+      <c r="K18" s="33"/>
+      <c r="L18" s="33"/>
+      <c r="M18" s="33"/>
+      <c r="N18" s="33"/>
+      <c r="O18" s="33"/>
+      <c r="P18" s="33"/>
       <c r="R18" s="26" t="str">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -2072,16 +2075,16 @@
         <v>14</v>
       </c>
       <c r="X18" s="7" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="Z18" t="str">
         <f t="shared" si="4"/>
         <v>MOV H040 K3Y20</v>
       </c>
     </row>
-    <row r="19" spans="4:26" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:26">
       <c r="D19" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="L19">
         <v>1</v>
@@ -2106,29 +2109,29 @@
         <v>15</v>
       </c>
       <c r="X19" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="Z19" t="str">
         <f t="shared" si="4"/>
         <v>MOV H010 K3Y20</v>
       </c>
     </row>
-    <row r="20" spans="4:26" x14ac:dyDescent="0.3">
-      <c r="D20" s="40" t="s">
-        <v>93</v>
-      </c>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-      <c r="H20" s="40"/>
-      <c r="I20" s="40"/>
-      <c r="J20" s="40"/>
-      <c r="K20" s="40"/>
-      <c r="L20" s="40"/>
-      <c r="M20" s="40"/>
-      <c r="N20" s="40"/>
-      <c r="O20" s="40"/>
-      <c r="P20" s="40"/>
+    <row r="20" spans="4:26">
+      <c r="D20" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
+      <c r="I20" s="33"/>
+      <c r="J20" s="33"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="33"/>
+      <c r="N20" s="33"/>
+      <c r="O20" s="33"/>
+      <c r="P20" s="33"/>
       <c r="R20" s="26" t="str">
         <f t="shared" ref="R20" si="5">IFERROR(VLOOKUP(E20*E$5+F20*F$5+G20*G$5+H20*H$5,$W$5:$X$19,2),"0")</f>
         <v>0</v>
@@ -2160,28 +2163,28 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:AC26"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
   <sheetData>
-    <row r="1" spans="2:29" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:29">
       <c r="Q1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="2" spans="2:29" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="2:29">
       <c r="C2" s="31" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="Q2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="2:29">
+      <c r="C3" s="31" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="C3" s="31" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="2:29" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:29" ht="17.25" thickBot="1"/>
+    <row r="5" spans="2:29">
       <c r="E5" s="9">
         <v>8</v>
       </c>
@@ -2234,10 +2237,10 @@
         <v>1</v>
       </c>
       <c r="AC5" s="30" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6" spans="2:29" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="2:29">
       <c r="E6" s="27"/>
       <c r="F6" s="28"/>
       <c r="G6" s="28"/>
@@ -2258,10 +2261,10 @@
         <v>2</v>
       </c>
       <c r="AC6" s="30" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="2:29" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="2:29">
       <c r="E7" s="27"/>
       <c r="F7" s="28"/>
       <c r="G7" s="28"/>
@@ -2282,15 +2285,15 @@
         <v>3</v>
       </c>
       <c r="AC7" s="30" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8" spans="2:29" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="2:29">
       <c r="B8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
@@ -2364,15 +2367,15 @@
         <v>4</v>
       </c>
       <c r="AC8" s="30" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="2:29" ht="17.25" thickBot="1">
       <c r="B9" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E9" s="15">
         <v>0</v>
@@ -2446,26 +2449,26 @@
         <v>5</v>
       </c>
       <c r="AC9" s="30" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="2:29" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="2:29">
       <c r="AB10" s="7">
         <v>6</v>
       </c>
       <c r="AC10" s="30" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="11" spans="2:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="2:29" ht="17.25" thickBot="1">
       <c r="AB11" s="7">
         <v>7</v>
       </c>
       <c r="AC11" s="30" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="12" spans="2:29" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="2:29">
       <c r="E12" s="18">
         <v>1</v>
       </c>
@@ -2538,10 +2541,10 @@
         <v>8</v>
       </c>
       <c r="AC12" s="30" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="13" spans="2:29" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="2:29">
       <c r="E13" s="21"/>
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
@@ -2582,10 +2585,10 @@
         <v>9</v>
       </c>
       <c r="AC13" s="30" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="14" spans="2:29" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="2:29">
       <c r="E14" s="21"/>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
@@ -2613,10 +2616,10 @@
         <v>10</v>
       </c>
       <c r="AC14" s="7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="15" spans="2:29" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="2:29">
       <c r="E15" s="21"/>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
@@ -2644,10 +2647,10 @@
         <v>11</v>
       </c>
       <c r="AC15" s="7" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="16" spans="2:29" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="2:29">
       <c r="E16" s="21"/>
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
@@ -2675,10 +2678,10 @@
         <v>12</v>
       </c>
       <c r="AC16" s="7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="17" spans="5:29" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="5:29">
       <c r="E17" s="21"/>
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
@@ -2706,10 +2709,10 @@
         <v>13</v>
       </c>
       <c r="AC17" s="7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="18" spans="5:29" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="5:29">
       <c r="E18" s="21"/>
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
@@ -2737,10 +2740,10 @@
         <v>14</v>
       </c>
       <c r="AC18" s="7" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="19" spans="5:29" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="5:29">
       <c r="E19" s="21"/>
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
@@ -2768,10 +2771,10 @@
         <v>15</v>
       </c>
       <c r="AC19" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="20" spans="5:29" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="5:29" ht="17.25" thickBot="1">
       <c r="E20" s="23"/>
       <c r="F20" s="24"/>
       <c r="G20" s="24"/>
@@ -2796,22 +2799,22 @@
       <c r="X20" s="26"/>
       <c r="Y20" s="26"/>
     </row>
-    <row r="23" spans="5:29" x14ac:dyDescent="0.3">
+    <row r="23" spans="5:29">
       <c r="W23" s="26"/>
       <c r="X23" s="26"/>
       <c r="Y23" s="26"/>
     </row>
-    <row r="24" spans="5:29" x14ac:dyDescent="0.3">
+    <row r="24" spans="5:29">
       <c r="W24" s="26"/>
       <c r="X24" s="26"/>
       <c r="Y24" s="26"/>
     </row>
-    <row r="25" spans="5:29" x14ac:dyDescent="0.3">
+    <row r="25" spans="5:29">
       <c r="W25" s="26"/>
       <c r="X25" s="26"/>
       <c r="Y25" s="26"/>
     </row>
-    <row r="26" spans="5:29" x14ac:dyDescent="0.3">
+    <row r="26" spans="5:29">
       <c r="W26" s="26"/>
       <c r="X26" s="26"/>
       <c r="Y26" s="26"/>

</xml_diff>